<commit_message>
feat: implement PDF batch processing and statistical analysis tools with comprehensive Architecture Decision Records.
</commit_message>
<xml_diff>
--- a/data/statistical_analysis_results.xlsx
+++ b/data/statistical_analysis_results.xlsx
@@ -1828,7 +1828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,20 +1844,10 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>평균 길이(단어)</t>
+          <t>평균 Overall Score</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>평균 다이어그램 수</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>평균 Overall Score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
         <is>
           <t>표준편차</t>
         </is>
@@ -1872,20 +1862,10 @@
       <c r="B2" t="n">
         <v>31</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>8,432</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
+      <c r="C2" t="n">
         <v>0.594</v>
       </c>
-      <c r="F2" t="n">
+      <c r="D2" t="n">
         <v>0.028</v>
       </c>
     </row>
@@ -1898,20 +1878,10 @@
       <c r="B3" t="n">
         <v>34</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>12,716</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
+      <c r="C3" t="n">
         <v>0.592</v>
       </c>
-      <c r="F3" t="n">
+      <c r="D3" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -1924,20 +1894,10 @@
       <c r="B4" t="n">
         <v>65</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>10,679</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="C4" t="n">
         <v>0.593</v>
       </c>
-      <c r="F4" t="n">
+      <c r="D4" t="n">
         <v>0.024</v>
       </c>
     </row>

</xml_diff>